<commit_message>
Update JLC sourcing BOM and five-board procurement workbooks
</commit_message>
<xml_diff>
--- a/engineering/JLCPCB_BOM_Stock_5_Boards.xlsx
+++ b/engineering/JLCPCB_BOM_Stock_5_Boards.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLC BOM" sheetId="1" r:id="R82858952baa843ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLC BOM" sheetId="1" r:id="R060aa2f789814a11"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -63,7 +63,9 @@
     </comment>
     <comment ref="I8" authorId="0">
       <text>
-        <t>Stock snapshot October 15, 2026: 850 at JLC. Five-board fitted need 10. Two parallel capacitors per PCB. 440 uF nominal bank; verify polarity, thermal/ripple performance and installed ESC transient behavior. Source: https://cart.jlcpcb.com/shoppingCart/smtGood/getComponentDetail?componentCode=C385885</t>
+        <r>
+          <t>Stock snapshot October 15, 2026: 850 at JLC. Five-board fitted need 10. Two parallel capacitors per PCB. 440 uF nominal bank; verify polarity, thermal/ripple performance and installed ESC transient behavior. Source: https://cart.jlcpcb.com/shoppingCart/smtGood/getComponentDetail?componentCode=C385885</t>
+        </r>
       </text>
     </comment>
     <comment ref="I9" authorId="0">
@@ -76,10 +78,7 @@
     </comment>
     <comment ref="I10" authorId="0">
       <text>
-        <r>
-          <t>Stock snapshot: October 15, 2026. Five-board fitted need: 10. Catalog loss estimate: 0. Actual JLC quote governs extras. Exact manufacturer/MPN match; assembly stock snapshot 2026-10-15.
-Source: https://cart.jlcpcb.com/shoppingCart/smtGood/getComponentDetail?componentCode=C3719750</t>
-        </r>
+        <t>Stock snapshot October 15, 2026: 3698 at JLC. Five-board fitted need 10. SMAJ24CA bidirectional SMA replacement, same nominal protection ratings; public JLC stock snapshot 3698, five-board fitted need 10 plus catalog loss 4. Source: https://cart.jlcpcb.com/shoppingCart/smtGood/getComponentDetail?componentCode=C28092</t>
       </text>
     </comment>
     <comment ref="I11" authorId="0">
@@ -260,10 +259,7 @@
     </comment>
     <comment ref="I33" authorId="0">
       <text>
-        <r>
-          <t>Stock snapshot: October 15, 2026. Five-board fitted need: 5. Catalog loss estimate: unconfirmed. Actual JLC quote governs extras. Exact JLC catalog match not verified; request global sourcing/consignment. Stock unavailable until JLC confirms receipt.
-Source: Exact catalog match unconfirmed.</t>
-        </r>
+        <t>Stock snapshot October 15, 2026: 2 at JLC. Five-board fitted need 5. Exact Vishay MPN match. Public JLC stock 2; five-board need 5, short 3. Global sourcing/private inventory required. Source: https://cart.jlcpcb.com/shoppingCart/smtGood/getComponentDetail?componentCode=C4265875</t>
       </text>
     </comment>
     <comment ref="I34" authorId="0">
@@ -292,7 +288,9 @@
     </comment>
     <comment ref="I37" authorId="0">
       <text>
-        <t>Stock snapshot October 15, 2026: 493 at JLC. Five-board fitted need 5. INA238 16-bit U2. Use updated INA238 firmware. Same DGS footprint and pinout as former INA228. Source: https://cart.jlcpcb.com/shoppingCart/smtGood/getComponentDetail?componentCode=C2868250</t>
+        <r>
+          <t>Stock snapshot October 15, 2026: 493 at JLC. Five-board fitted need 5. INA238 16-bit U2. Use updated INA238 firmware. Same DGS footprint and pinout as former INA228. Source: https://cart.jlcpcb.com/shoppingCart/smtGood/getComponentDetail?componentCode=C2868250</t>
+        </r>
       </text>
     </comment>
     <comment ref="I38" authorId="0">
@@ -937,19 +935,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="E10" s="8" t="str">
-        <x:v>Bourns</x:v>
+        <x:v>RUILON</x:v>
       </x:c>
       <x:c r="F10" s="8" t="str">
         <x:v>SMAJ24CA</x:v>
       </x:c>
       <x:c r="G10" s="8" t="str">
-        <x:v>C3719750</x:v>
+        <x:v>C28092</x:v>
       </x:c>
       <x:c r="H10" s="12" t="n">
-        <x:v>0</x:v>
+        <x:v>3698</x:v>
       </x:c>
       <x:c r="I10" s="8" t="str">
-        <x:v>Short stock</x:v>
+        <x:v>Stock sufficient</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="39" customHeight="1">
@@ -1597,10 +1595,14 @@
       <x:c r="F33" s="9" t="str">
         <x:v>CRCW25121K00FKEGHP</x:v>
       </x:c>
-      <x:c r="G33" s="9" t="str"/>
-      <x:c r="H33" s="13"/>
+      <x:c r="G33" s="9" t="str">
+        <x:v>C4265875</x:v>
+      </x:c>
+      <x:c r="H33" s="13" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="I33" s="9" t="str">
-        <x:v>Unconfirmed</x:v>
+        <x:v>Short stock</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="39" customHeight="1">
@@ -1812,6 +1814,6 @@
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Unconfirmed"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda75ad0aa2524c08"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d3c82fbbfb94ed6"/>
 </x:worksheet>
 </file>
</xml_diff>